<commit_message>
Replace ans.fr.nos dependency with ans.fr.terminologies
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com> 7d2a0e2af4c793b5df5fce306b2316e2695dbc78
</commit_message>
<xml_diff>
--- a/nr-prepare-release/ig/ConceptMap-mos-cdl.xlsx
+++ b/nr-prepare-release/ig/ConceptMap-mos-cdl.xlsx
@@ -65,7 +65,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-20T08:30:08+00:00</t>
+    <t>2026-07-20T08:39:03+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -83,7 +83,7 @@
     <t>Jurisdiction</t>
   </si>
   <si>
-    <t>FRANCE</t>
+    <t>France (la)</t>
   </si>
   <si>
     <t>Description</t>

</xml_diff>